<commit_message>
Logs para experimentación red de 4 nodos
</commit_message>
<xml_diff>
--- a/Casos/problema_chatGPT/resultados_excel/instancia2.xlsx
+++ b/Casos/problema_chatGPT/resultados_excel/instancia2.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Laura\OneDrive - Universidad Politécnica de Madrid\optimal_power_flow\github\Casos\problema_chatGPT\resultados_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3587530-488B-45A3-84FB-E2B147E83AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD8B2EC-DD86-44AF-B293-B5AA257E125F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{52D9C27D-0EF6-DD41-9728-0267E68F7539}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Concepto</t>
   </si>
@@ -60,13 +71,7 @@
     <t>Desviación típica del coste por instancia</t>
   </si>
   <si>
-    <t>MINLP</t>
-  </si>
-  <si>
-    <t>Coste de generación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se encuentra la solución óptima con el PSO. El MINLP es mejor. Probar a hacerlo sin el análisis múltiple. </t>
+    <t>Coste de generación con MINLP</t>
   </si>
 </sst>
 </file>
@@ -418,13 +423,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF0E20E-E4D8-9B45-9C94-E89B574F109C}">
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.4140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -432,7 +437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -440,7 +445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -448,7 +453,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -456,70 +461,60 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5">
-        <v>264.74060001373289</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+        <v>553.40840001106267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>14.686216221223701</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+        <v>136.74241397150001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>7</v>
       </c>
       <c r="B7">
-        <v>2385.7166075906985</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3230.014850724207</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>8</v>
       </c>
       <c r="B8">
-        <v>2389.7144476540784</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3335.9990934551361</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
       <c r="B9">
-        <v>2382.4426508829856</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3181.0169272619869</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
       <c r="B10">
-        <v>3.2049661031842116</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+        <v>70.916906617219013</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>2220</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>13</v>
+      <c r="B12">
+        <v>3181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>